<commit_message>
Dedupe account-lockout test cases (026-031 -> TC-LP-026); 17 fail -> 12
Per-role lockout cases identical after Role column dropped; merged to one.
Totals now 94 cases / 82 PASS / 12 FAIL (87.2%), 1:1 with 12 bugs.
Updated xlsx, deck, README.
</commit_message>
<xml_diff>
--- a/SauceDemo (Test Cases).xlsx
+++ b/SauceDemo (Test Cases).xlsx
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Verify account lockout on multiple failed attempts</t>
+          <t>Verify account lockout on multiple failed attempts (semua user role)</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1548,220 +1548,15 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TC-LP-027</t>
+          <t>TC-LP-032</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Verify account lockout on multiple failed attempts</t>
+          <t>Verify login across multiple browsers</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>Hasil tidak sesuai — lihat Defect Report</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>TC-LP-028</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Verify account lockout on multiple failed attempts</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Hasil tidak sesuai — lihat Defect Report</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>TC-LP-029</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Verify account lockout on multiple failed attempts</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Hasil tidak sesuai — lihat Defect Report</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>TC-LP-030</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Verify account lockout on multiple failed attempts</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>Hasil tidak sesuai — lihat Defect Report</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>TC-LP-031</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Verify account lockout on multiple failed attempts</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Hasil tidak sesuai — lihat Defect Report</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>TC-LP-032</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Verify login across multiple browsers</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Enter valid credentials. 
@@ -1769,39 +1564,39 @@
 4. Repeat on different browsers</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>User is successfully logged in and redirected to homepage</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>User is successfully logged in and redirected to homepage</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>TC-LP-033</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Verify login across multiple browsers</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Enter valid credentials
@@ -1809,39 +1604,39 @@
 4. Repeat on different browsers</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Error message appears: "Sorry, this user has been locked out"</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>Erros message: Epic sadface: Sorry, this user has been locked out.</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>TC-LP-034</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Verify login across multiple browsers</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Enter valid credentials
@@ -1849,39 +1644,39 @@
 4. Repeat on different browsers</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>User logs in successfully, but UI may have bugs (e.g., broken images, misaligned elements)</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>User logs in successfully, but UI may have bugs (e.g., broken images, misaligned elements)</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>TC-LP-035</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Verify login across multiple browsers</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Enter valid credentials
@@ -1889,39 +1684,39 @@
 4. Repeat on different browsers</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Login process is significantly slower compared to other users</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>Login process is significantly slower compared to other users</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>TC-LP-036</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Verify login across multiple browsers</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Enter valid credentials
@@ -1929,39 +1724,39 @@
 4. Repeat on different browsers</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>System may behave unexpectedly (e.g., crash, show an error)</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>System behaves unexpectedly (e.g., crash, show an error)</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>TC-LP-037</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Verify login across multiple browsers</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Enter valid credentials
@@ -1969,39 +1764,39 @@
 4. Repeat on different browsers</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>User logs in successfully, but UI elements may appear distorted</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>User logs in successfully, but UI elements appear distorted</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>TC-LP-038</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Verify login on mobile devices</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Open mobile browser
@@ -2009,39 +1804,39 @@
 4. Click Login</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>User is successfully logged in and redirected to homepage</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>User is successfully logged in and redirected to homepage</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>TC-LP-039</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Verify login on mobile devices</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Open mobile browser
@@ -2049,39 +1844,39 @@
 4. Click Login</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>Error message appears: "Sorry, this user has been locked out"</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>Erros message: Epic sadface: Sorry, this user has been locked out.</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>TC-LP-040</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Verify login on mobile devices</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Open mobile browser
@@ -2089,39 +1884,39 @@
 4. Click Login</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>User logs in successfully, but UI may have bugs (e.g., broken images, misaligned elements)</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>User logs in successfully, but UI may have bugs (e.g., broken images, misaligned elements)</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>TC-LP-041</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>Verify login on mobile devices</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Open mobile browser
@@ -2129,39 +1924,39 @@
 4. Click Login</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>Login process is significantly slower compared to other users</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>Login process is significantly slower compared to other users</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>TC-LP-042</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Verify login on mobile devices</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Open mobile browser
@@ -2169,39 +1964,39 @@
 4. Click Login</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>System may behave unexpectedly (e.g., crash, show an error)</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>System behaves unexpectedly (e.g., crash, show an error)</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>TC-LP-043</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Verify login on mobile devices</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Open mobile browser
@@ -2209,65 +2004,110 @@
 4. Click Login</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>User logs in successfully, but UI elements may appear distorted</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>User logs in successfully, but UI elements appear distorted</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>TC-LP-044</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Verify password field masking</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>1. Go to "https://www.saucedemo.com/"
 2. Enter password
 3. Check if characters are masked</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Password char must be masked</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Password char is masked</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>Sesuai dengan expected result</t>
-        </is>
-      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Sesuai dengan expected result</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n"/>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="4" t="n"/>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n"/>
+      <c r="B43" s="4" t="n"/>
+      <c r="C43" s="4" t="n"/>
+      <c r="D43" s="4" t="n"/>
+      <c r="E43" s="4" t="n"/>
+      <c r="F43" s="5" t="n"/>
+      <c r="G43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n"/>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>